<commit_message>
COHORT_19 and Echo files
My computer had a more updated version of COHORT_19.csv than the parent repository had so I replaced the version on the parent repository with this one. There were two EchoMRI files that I needed to add since they weren't in the original repository
</commit_message>
<xml_diff>
--- a/data/echoMRI/Kotz04292026.xlsx
+++ b/data/echoMRI/Kotz04292026.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
   <workbookPr backupFile="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carosandovalcab/Documents/GitHub/data/data/echoMRI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/laurenmichels/Documents/GitHub/data/data/echoMRI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92EACD81-DD31-754D-A559-C91A44E826F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{56AB7DFA-2D0E-8C44-BB42-5247248128BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="44800" windowHeight="25200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17500" yWindow="680" windowWidth="24480" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtractedScans" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExtractedScans">ExtractedScans!$A$1:$J$18</definedName>
+    <definedName name="ExtractedScans">ExtractedScans!$A$1:$J$8</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>RecNumber</t>
   </si>
@@ -55,106 +55,46 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>9432</t>
-  </si>
-  <si>
-    <t>9433</t>
-  </si>
-  <si>
-    <t>9437</t>
-  </si>
-  <si>
-    <t>9441</t>
-  </si>
-  <si>
-    <t>9449</t>
-  </si>
-  <si>
-    <t>9451</t>
-  </si>
-  <si>
-    <t>9452</t>
-  </si>
-  <si>
-    <t>9454</t>
-  </si>
-  <si>
-    <t>9455</t>
-  </si>
-  <si>
-    <t>9436</t>
-  </si>
-  <si>
-    <t>9438</t>
-  </si>
-  <si>
-    <t>9439</t>
-  </si>
-  <si>
-    <t>9443</t>
-  </si>
-  <si>
-    <t>9444</t>
-  </si>
-  <si>
-    <t>9450</t>
-  </si>
-  <si>
-    <t>9453</t>
-  </si>
-  <si>
-    <t>9456</t>
-  </si>
-  <si>
-    <t>11:23:57 Apr 29, 2026; 27; ems</t>
-  </si>
-  <si>
-    <t>11:25:04 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:26:39 Apr 29, 2026; 27; ems</t>
-  </si>
-  <si>
-    <t>11:27:50 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:29:10 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:30:30 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:31:39 Apr 29, 2026; 27; ems</t>
-  </si>
-  <si>
-    <t>11:32:54 Apr 29, 2026; 27; ems</t>
-  </si>
-  <si>
-    <t>11:34:17 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:35:27 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:36:49 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:38:29 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:39:48 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:41:01 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:42:16 Apr 29, 2026; 32; ems</t>
-  </si>
-  <si>
-    <t>11:43:37 Apr 29, 2026; 31; ems</t>
-  </si>
-  <si>
-    <t>11:45:00 Apr 29, 2026; 31; ems</t>
+    <t>3748</t>
+  </si>
+  <si>
+    <t>3749</t>
+  </si>
+  <si>
+    <t>3750</t>
+  </si>
+  <si>
+    <t>3752</t>
+  </si>
+  <si>
+    <t>3753</t>
+  </si>
+  <si>
+    <t>3751</t>
+  </si>
+  <si>
+    <t>3747</t>
+  </si>
+  <si>
+    <t>10:45:58 Apr 29, 2026; 31; ems</t>
+  </si>
+  <si>
+    <t>10:47:11 Apr 29, 2026; 31; ems</t>
+  </si>
+  <si>
+    <t>10:48:27 Apr 29, 2026; 31; ems</t>
+  </si>
+  <si>
+    <t>10:49:49 Apr 29, 2026; 27; ems</t>
+  </si>
+  <si>
+    <t>10:51:04 Apr 29, 2026; 31; ems</t>
+  </si>
+  <si>
+    <t>10:52:30 Apr 29, 2026; 27; ems</t>
+  </si>
+  <si>
+    <t>10:53:43 Apr 29, 2026; 31; ems</t>
   </si>
 </sst>
 </file>
@@ -493,10 +433,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13"/>
   <cols>
-    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="7" max="7" width="27.3984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -536,13 +476,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C2">
-        <v>9.75</v>
+        <v>14.53</v>
       </c>
       <c r="D2">
-        <v>27.67</v>
+        <v>22.74</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -551,13 +491,13 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>37.58</v>
+        <v>36.74</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -565,13 +505,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3">
-        <v>10.85</v>
+        <v>21.57</v>
       </c>
       <c r="D3">
-        <v>28.28</v>
+        <v>23.58</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -580,13 +520,13 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>40.21</v>
+        <v>44.14</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -594,13 +534,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4">
-        <v>26.33</v>
+        <v>12.47</v>
       </c>
       <c r="D4">
-        <v>43.67</v>
+        <v>20.440000000000001</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -609,13 +549,13 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="I4">
-        <v>69.98</v>
+        <v>32.43</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -623,13 +563,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5">
-        <v>11.26</v>
+        <v>21.33</v>
       </c>
       <c r="D5">
-        <v>37.93</v>
+        <v>22.58</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -638,13 +578,13 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H5">
         <v>1</v>
       </c>
       <c r="I5">
-        <v>48.22</v>
+        <v>43.06</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -652,13 +592,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>2.21</v>
+        <v>16.47</v>
       </c>
       <c r="D6">
-        <v>27.07</v>
+        <v>23.07</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -667,13 +607,13 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6">
-        <v>30.15</v>
+        <v>38.950000000000003</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -681,13 +621,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C7">
-        <v>10.119999999999999</v>
+        <v>16.21</v>
       </c>
       <c r="D7">
-        <v>32.6</v>
+        <v>23.84</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -696,13 +636,13 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7">
-        <v>41.93</v>
+        <v>39.43</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -710,13 +650,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8">
-        <v>11.53</v>
+        <v>19.23</v>
       </c>
       <c r="D8">
-        <v>30.8</v>
+        <v>23.52</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -725,303 +665,13 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>42.39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9">
-        <v>16.559999999999999</v>
-      </c>
-      <c r="D9">
-        <v>39.78</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9" t="s">
-        <v>34</v>
-      </c>
-      <c r="H9">
-        <v>1</v>
-      </c>
-      <c r="I9">
-        <v>56.13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10">
-        <v>12.16</v>
-      </c>
-      <c r="D10">
-        <v>27.99</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10" t="s">
-        <v>35</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10">
-        <v>39.43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11">
-        <v>9.34</v>
-      </c>
-      <c r="D11">
-        <v>26.86</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11" t="s">
-        <v>36</v>
-      </c>
-      <c r="H11">
-        <v>1</v>
-      </c>
-      <c r="I11">
-        <v>36.17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12">
-        <v>8.32</v>
-      </c>
-      <c r="D12">
-        <v>30.63</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12" t="s">
-        <v>37</v>
-      </c>
-      <c r="H12">
-        <v>1</v>
-      </c>
-      <c r="I12">
-        <v>39.630000000000003</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13">
-        <v>10.98</v>
-      </c>
-      <c r="D13">
-        <v>31.21</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13" t="s">
-        <v>38</v>
-      </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-      <c r="I13">
         <v>42.03</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14">
-        <v>11.93</v>
-      </c>
-      <c r="D14">
-        <v>25.86</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14" t="s">
-        <v>39</v>
-      </c>
-      <c r="H14">
-        <v>1</v>
-      </c>
-      <c r="I14">
-        <v>38.21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15">
-        <v>1.98</v>
-      </c>
-      <c r="D15">
-        <v>25.78</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15" t="s">
-        <v>40</v>
-      </c>
-      <c r="H15">
-        <v>1</v>
-      </c>
-      <c r="I15">
-        <v>29.33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16">
-        <v>5.12</v>
-      </c>
-      <c r="D16">
-        <v>30.29</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16" t="s">
-        <v>41</v>
-      </c>
-      <c r="H16">
-        <v>1</v>
-      </c>
-      <c r="I16">
-        <v>35.44</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17">
-        <v>8.69</v>
-      </c>
-      <c r="D17">
-        <v>32.020000000000003</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17" t="s">
-        <v>42</v>
-      </c>
-      <c r="H17">
-        <v>1</v>
-      </c>
-      <c r="I17">
-        <v>41.25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18">
-        <v>3.08</v>
-      </c>
-      <c r="D18">
-        <v>29.8</v>
-      </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
-      <c r="G18" t="s">
-        <v>43</v>
-      </c>
-      <c r="H18">
-        <v>1</v>
-      </c>
-      <c r="I18">
-        <v>34.340000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>